<commit_message>
adding instability for Rb and iodine
</commit_message>
<xml_diff>
--- a/linewidth list.xlsx
+++ b/linewidth list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\Jonathan\kuliah\kurikuler\semester 7\proposal TA\Weekly progress\Bi-SAS-for-Optical-Clock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{48429F16-08BE-48D4-9A35-5E42FFB329CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB1C34B-573E-47E3-BDE1-CFCBDBC0FE35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="23040" windowHeight="12240" activeTab="3" xr2:uid="{A9525EA0-AC80-4C32-9AB0-7DB911FE4C9F}"/>
+    <workbookView xWindow="108" yWindow="36" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{A9525EA0-AC80-4C32-9AB0-7DB911FE4C9F}"/>
   </bookViews>
   <sheets>
     <sheet name="F'=0" sheetId="1" r:id="rId1"/>

</xml_diff>